<commit_message>
docs: Add summary comments and notes into experiments.xlsx
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -6314,7 +6314,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H2" s="38" t="n"/>
+      <c r="H2" s="38" t="inlineStr">
+        <is>
+          <t>Baseline M-base on dinh qua 3 seed, val_macro_f1 quanh 0.8410, vuot xa moc doan da so.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="20">
       <c r="A3" s="31" t="inlineStr">
@@ -6346,7 +6350,11 @@
         <f>IF(C3&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H3" s="38" t="n"/>
+      <c r="H3" s="38" t="inlineStr">
+        <is>
+          <t>CE vuot troi so voi MSE (+0.1457 val_macro_f1) nho gradient khong bi bao hoa khi sai so lon.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="20">
       <c r="A4" s="31" t="inlineStr">
@@ -6378,7 +6386,11 @@
         <f>IF(C4&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H4" s="38" t="n"/>
+      <c r="H4" s="38" t="inlineStr">
+        <is>
+          <t>Adam lr=1e-3 dat cao nhat (0.8462); Momentum giup SGD tang manh tu 0.6975 len 0.8389.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="20">
       <c r="A5" s="31" t="inlineStr">
@@ -6410,7 +6422,11 @@
         <f>IF(C5&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H5" s="38" t="n"/>
+      <c r="H5" s="38" t="inlineStr">
+        <is>
+          <t>M-deep dat 0.8621 va M-wide dat 0.8594; batch 128 hoi tu nhanh hon batch 2048.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="20">
       <c r="A6" s="31" t="inlineStr">
@@ -6442,7 +6458,11 @@
         <f>IF(C6&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H6" s="38" t="n"/>
+      <c r="H6" s="38" t="inlineStr">
+        <is>
+          <t>Mo hinh chua qua khop (gap val-train chi 0.02) nen dropout lam giam nang luc bieu dien.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="20">
       <c r="A7" s="31" t="inlineStr">
@@ -6474,7 +6494,11 @@
         <f>IF(C7&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H7" s="38" t="n"/>
+      <c r="H7" s="38" t="inlineStr">
+        <is>
+          <t>Clipping c=1.0 cuu mo hinh khoi dao dong manh va mat on dinh khi learning rate cao (lr=0.8).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="20">
       <c r="A8" s="31" t="inlineStr">
@@ -6506,7 +6530,11 @@
         <f>IF(C8&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H8" s="38" t="n"/>
+      <c r="H8" s="38" t="inlineStr">
+        <is>
+          <t>FP16 Autocast hoat dong on dinh voi GradScaler, tiet kiem 50% VRAM tren GPU.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="20">
       <c r="A9" s="31" t="inlineStr">
@@ -6538,7 +6566,11 @@
         <f>IF(C9&gt;0,"Có","Chưa")</f>
         <v/>
       </c>
-      <c r="H9" s="38" t="n"/>
+      <c r="H9" s="38" t="inlineStr">
+        <is>
+          <t>Khoi tao He duy tri tot nhat phuong sai cho ReLU; Zeros that bai hoan toan do doi xung.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="20">
       <c r="A10" s="31" t="inlineStr">
@@ -6571,7 +6603,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H10" s="38" t="n"/>
+      <c r="H10" s="38" t="inlineStr">
+        <is>
+          <t>Cau hinh toi uu Adam lr=1e-3 dat eval macro-F1 = 0.8515, vuot moc baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="20">
       <c r="A11" s="31" t="inlineStr">

</xml_diff>